<commit_message>
Rearrange capacity tiers; clean up stale files
Capacity changes (shelter_capacity.py):
- New thresholds: ≤9p→6, ≤16p→12, ≤24p→20, ≤40p→30, >40p→50
- 12p is now the most common tier (182 shelters, 57%)
- 6p used for genuinely low-traffic rural roads (13 shelters)
- Total capital cost: ₪45.1M (was ₪56M); 10-year: ₪99.8M

Repo cleanup:
- Remove stale files: export_datasets.py, road_shelters_traffic.py,
  shelter_qa.py, shelters_priority_final.html, shelter_points_priority.pkl
- Add .gitignore: DS_Store, __pycache__, *.pkl, *.bak, old road_shelters_* outputs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/budget_shelters_v2.xlsx
+++ b/budget_shelters_v2.xlsx
@@ -558,7 +558,7 @@
         <v>73000</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D6" s="6">
         <f>B6*C6</f>
@@ -573,7 +573,7 @@
         <v>100000</v>
       </c>
       <c r="C7" t="n">
-        <v>29</v>
+        <v>182</v>
       </c>
       <c r="D7" s="6">
         <f>B7*C7</f>
@@ -588,7 +588,7 @@
         <v>150000</v>
       </c>
       <c r="C8" t="n">
-        <v>181</v>
+        <v>31</v>
       </c>
       <c r="D8" s="6">
         <f>B8*C8</f>
@@ -603,7 +603,7 @@
         <v>200000</v>
       </c>
       <c r="C9" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="D9" s="6">
         <f>B9*C9</f>
@@ -618,7 +618,7 @@
         <v>250000</v>
       </c>
       <c r="C10" t="n">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="D10" s="6">
         <f>B10*C10</f>
@@ -875,10 +875,10 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I3" s="13" t="n">
         <v>8000</v>
@@ -922,10 +922,10 @@
         </is>
       </c>
       <c r="G4" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H4" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I4" s="17" t="n">
         <v>9000</v>
@@ -969,10 +969,10 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I5" s="13" t="n">
         <v>20000</v>
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="G6" s="14" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I6" s="17" t="n">
         <v>20000</v>
@@ -1063,10 +1063,10 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I7" s="13" t="n">
         <v>13000</v>
@@ -1157,10 +1157,10 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I9" s="13" t="n">
         <v>4000</v>
@@ -1204,10 +1204,10 @@
         </is>
       </c>
       <c r="G10" s="14" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I10" s="17" t="n">
         <v>8000</v>
@@ -1251,10 +1251,10 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I11" s="13" t="n">
         <v>9000</v>
@@ -1298,10 +1298,10 @@
         </is>
       </c>
       <c r="G12" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I12" s="17" t="n">
         <v>8000</v>
@@ -1345,10 +1345,10 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I13" s="13" t="n">
         <v>8000</v>
@@ -1486,10 +1486,10 @@
         </is>
       </c>
       <c r="G16" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I16" s="17" t="n">
         <v>8000</v>
@@ -1627,10 +1627,10 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I19" s="13" t="n">
         <v>8000</v>
@@ -1721,10 +1721,10 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I21" s="13" t="n">
         <v>8000</v>
@@ -1768,10 +1768,10 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H22" s="16" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I22" s="17" t="n">
         <v>8000</v>
@@ -1815,10 +1815,10 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I23" s="13" t="n">
         <v>8000</v>
@@ -1909,10 +1909,10 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I25" s="13" t="n">
         <v>8000</v>
@@ -1956,10 +1956,10 @@
         </is>
       </c>
       <c r="G26" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H26" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I26" s="17" t="n">
         <v>8000</v>
@@ -2003,10 +2003,10 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I27" s="13" t="n">
         <v>8000</v>
@@ -2097,10 +2097,10 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I29" s="13" t="n">
         <v>8000</v>
@@ -2285,10 +2285,10 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I33" s="13" t="n">
         <v>8000</v>
@@ -2332,10 +2332,10 @@
         </is>
       </c>
       <c r="G34" s="14" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H34" s="16" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I34" s="17" t="n">
         <v>8000</v>
@@ -2379,10 +2379,10 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I35" s="13" t="n">
         <v>8000</v>
@@ -2612,10 +2612,10 @@
         </is>
       </c>
       <c r="G40" s="14" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H40" s="16" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I40" s="17" t="n">
         <v>20000</v>
@@ -2659,10 +2659,10 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I41" s="13" t="n">
         <v>8000</v>
@@ -2800,10 +2800,10 @@
         </is>
       </c>
       <c r="G44" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H44" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I44" s="17" t="n">
         <v>8000</v>
@@ -2847,10 +2847,10 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I45" s="13" t="n">
         <v>8000</v>
@@ -2894,10 +2894,10 @@
         </is>
       </c>
       <c r="G46" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H46" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I46" s="17" t="n">
         <v>8000</v>
@@ -2941,10 +2941,10 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I47" s="13" t="n">
         <v>8000</v>
@@ -2988,10 +2988,10 @@
         </is>
       </c>
       <c r="G48" s="14" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H48" s="16" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I48" s="17" t="n">
         <v>8000</v>
@@ -3035,10 +3035,10 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I49" s="13" t="n">
         <v>8000</v>
@@ -3082,10 +3082,10 @@
         </is>
       </c>
       <c r="G50" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H50" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I50" s="17" t="n">
         <v>9000</v>
@@ -3176,10 +3176,10 @@
         </is>
       </c>
       <c r="G52" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H52" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I52" s="17" t="n">
         <v>8500</v>
@@ -3223,10 +3223,10 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H53" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I53" s="13" t="n">
         <v>9000</v>
@@ -3317,10 +3317,10 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H55" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I55" s="13" t="n">
         <v>20000</v>
@@ -3411,10 +3411,10 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H57" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I57" s="13" t="n">
         <v>8500</v>
@@ -3458,10 +3458,10 @@
         </is>
       </c>
       <c r="G58" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H58" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I58" s="17" t="n">
         <v>8000</v>
@@ -3505,10 +3505,10 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H59" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I59" s="13" t="n">
         <v>8000</v>
@@ -3597,10 +3597,10 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H61" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I61" s="13" t="n">
         <v>8000</v>
@@ -3644,10 +3644,10 @@
         </is>
       </c>
       <c r="G62" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H62" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I62" s="17" t="n">
         <v>9000</v>
@@ -3877,10 +3877,10 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H67" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I67" s="13" t="n">
         <v>8000</v>
@@ -3924,10 +3924,10 @@
         </is>
       </c>
       <c r="G68" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H68" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I68" s="17" t="n">
         <v>8000</v>
@@ -3971,10 +3971,10 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H69" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I69" s="13" t="n">
         <v>8000</v>
@@ -4065,10 +4065,10 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H71" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I71" s="13" t="n">
         <v>8000</v>
@@ -4112,10 +4112,10 @@
         </is>
       </c>
       <c r="G72" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H72" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I72" s="17" t="n">
         <v>8000</v>
@@ -4204,10 +4204,10 @@
         </is>
       </c>
       <c r="G74" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H74" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I74" s="17" t="n">
         <v>8000</v>
@@ -4345,10 +4345,10 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H77" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I77" s="13" t="n">
         <v>8000</v>
@@ -4392,10 +4392,10 @@
         </is>
       </c>
       <c r="G78" s="14" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H78" s="16" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I78" s="17" t="n">
         <v>18000</v>
@@ -4439,10 +4439,10 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H79" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I79" s="13" t="n">
         <v>20000</v>
@@ -4486,10 +4486,10 @@
         </is>
       </c>
       <c r="G80" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H80" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I80" s="17" t="n">
         <v>8000</v>
@@ -4533,10 +4533,10 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H81" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I81" s="13" t="n">
         <v>8000</v>
@@ -4580,10 +4580,10 @@
         </is>
       </c>
       <c r="G82" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H82" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I82" s="17" t="n">
         <v>8000</v>
@@ -4627,10 +4627,10 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H83" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I83" s="13" t="n">
         <v>8000</v>
@@ -4766,10 +4766,10 @@
         </is>
       </c>
       <c r="G86" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H86" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I86" s="17" t="n">
         <v>8000</v>
@@ -4813,10 +4813,10 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H87" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I87" s="13" t="n">
         <v>8000</v>
@@ -5001,10 +5001,10 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H91" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I91" s="13" t="n">
         <v>8000</v>
@@ -5048,10 +5048,10 @@
         </is>
       </c>
       <c r="G92" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H92" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I92" s="17" t="n">
         <v>8000</v>
@@ -5142,10 +5142,10 @@
         </is>
       </c>
       <c r="G94" s="14" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H94" s="16" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I94" s="17" t="n">
         <v>18000</v>
@@ -5189,10 +5189,10 @@
         </is>
       </c>
       <c r="G95" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H95" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I95" s="13" t="n">
         <v>8000</v>
@@ -5283,10 +5283,10 @@
         </is>
       </c>
       <c r="G97" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H97" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I97" s="13" t="n">
         <v>8000</v>
@@ -5377,10 +5377,10 @@
         </is>
       </c>
       <c r="G99" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H99" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I99" s="13" t="n">
         <v>8000</v>
@@ -5424,10 +5424,10 @@
         </is>
       </c>
       <c r="G100" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H100" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I100" s="17" t="n">
         <v>8000</v>
@@ -5565,10 +5565,10 @@
         </is>
       </c>
       <c r="G103" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H103" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I103" s="13" t="n">
         <v>8000</v>
@@ -5612,10 +5612,10 @@
         </is>
       </c>
       <c r="G104" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H104" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I104" s="17" t="n">
         <v>8000</v>
@@ -5659,10 +5659,10 @@
         </is>
       </c>
       <c r="G105" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H105" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I105" s="13" t="n">
         <v>8000</v>
@@ -5845,10 +5845,10 @@
         </is>
       </c>
       <c r="G109" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H109" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I109" s="13" t="n">
         <v>8000</v>
@@ -5937,10 +5937,10 @@
         </is>
       </c>
       <c r="G111" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H111" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I111" s="13" t="n">
         <v>8000</v>
@@ -5984,10 +5984,10 @@
         </is>
       </c>
       <c r="G112" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H112" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I112" s="17" t="n">
         <v>11000</v>
@@ -6078,10 +6078,10 @@
         </is>
       </c>
       <c r="G114" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H114" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I114" s="17" t="n">
         <v>8000</v>
@@ -6125,10 +6125,10 @@
         </is>
       </c>
       <c r="G115" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H115" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I115" s="13" t="n">
         <v>8000</v>
@@ -6172,10 +6172,10 @@
         </is>
       </c>
       <c r="G116" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H116" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I116" s="17" t="n">
         <v>8000</v>
@@ -6219,10 +6219,10 @@
         </is>
       </c>
       <c r="G117" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H117" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I117" s="13" t="n">
         <v>4000</v>
@@ -6266,10 +6266,10 @@
         </is>
       </c>
       <c r="G118" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H118" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I118" s="17" t="n">
         <v>8000</v>
@@ -6360,10 +6360,10 @@
         </is>
       </c>
       <c r="G120" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H120" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I120" s="17" t="n">
         <v>8000</v>
@@ -6407,10 +6407,10 @@
         </is>
       </c>
       <c r="G121" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H121" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I121" s="13" t="n">
         <v>4000</v>
@@ -6454,10 +6454,10 @@
         </is>
       </c>
       <c r="G122" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H122" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I122" s="17" t="n">
         <v>7000</v>
@@ -6501,10 +6501,10 @@
         </is>
       </c>
       <c r="G123" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H123" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I123" s="13" t="n">
         <v>8000</v>
@@ -6548,10 +6548,10 @@
         </is>
       </c>
       <c r="G124" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H124" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I124" s="17" t="n">
         <v>8000</v>
@@ -6642,10 +6642,10 @@
         </is>
       </c>
       <c r="G126" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H126" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I126" s="17" t="n">
         <v>8000</v>
@@ -6689,10 +6689,10 @@
         </is>
       </c>
       <c r="G127" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H127" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I127" s="13" t="n">
         <v>8000</v>
@@ -6736,10 +6736,10 @@
         </is>
       </c>
       <c r="G128" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H128" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I128" s="17" t="n">
         <v>8000</v>
@@ -6830,10 +6830,10 @@
         </is>
       </c>
       <c r="G130" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H130" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I130" s="17" t="n">
         <v>8000</v>
@@ -6877,10 +6877,10 @@
         </is>
       </c>
       <c r="G131" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H131" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I131" s="13" t="n">
         <v>8000</v>
@@ -6924,10 +6924,10 @@
         </is>
       </c>
       <c r="G132" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H132" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I132" s="17" t="n">
         <v>8000</v>
@@ -7018,10 +7018,10 @@
         </is>
       </c>
       <c r="G134" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H134" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I134" s="17" t="n">
         <v>8000</v>
@@ -7112,10 +7112,10 @@
         </is>
       </c>
       <c r="G136" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H136" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I136" s="17" t="n">
         <v>8000</v>
@@ -7159,10 +7159,10 @@
         </is>
       </c>
       <c r="G137" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H137" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I137" s="13" t="n">
         <v>8000</v>
@@ -7206,10 +7206,10 @@
         </is>
       </c>
       <c r="G138" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H138" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I138" s="17" t="n">
         <v>8000</v>
@@ -7253,10 +7253,10 @@
         </is>
       </c>
       <c r="G139" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H139" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I139" s="13" t="n">
         <v>20000</v>
@@ -7300,10 +7300,10 @@
         </is>
       </c>
       <c r="G140" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H140" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I140" s="17" t="n">
         <v>8000</v>
@@ -7441,10 +7441,10 @@
         </is>
       </c>
       <c r="G143" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H143" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I143" s="13" t="n">
         <v>8000</v>
@@ -7488,10 +7488,10 @@
         </is>
       </c>
       <c r="G144" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H144" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I144" s="17" t="n">
         <v>8000</v>
@@ -7535,10 +7535,10 @@
         </is>
       </c>
       <c r="G145" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H145" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I145" s="13" t="n">
         <v>8000</v>
@@ -7582,10 +7582,10 @@
         </is>
       </c>
       <c r="G146" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H146" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I146" s="17" t="n">
         <v>8000</v>
@@ -7629,10 +7629,10 @@
         </is>
       </c>
       <c r="G147" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H147" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I147" s="13" t="n">
         <v>19000</v>
@@ -7723,10 +7723,10 @@
         </is>
       </c>
       <c r="G149" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H149" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I149" s="13" t="n">
         <v>8000</v>
@@ -7817,10 +7817,10 @@
         </is>
       </c>
       <c r="G151" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H151" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I151" s="13" t="n">
         <v>8000</v>
@@ -7909,10 +7909,10 @@
         </is>
       </c>
       <c r="G153" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H153" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I153" s="13" t="n">
         <v>8000</v>
@@ -8003,10 +8003,10 @@
         </is>
       </c>
       <c r="G155" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H155" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I155" s="13" t="n">
         <v>8000</v>
@@ -8097,10 +8097,10 @@
         </is>
       </c>
       <c r="G157" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H157" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I157" s="13" t="n">
         <v>8000</v>
@@ -8144,10 +8144,10 @@
         </is>
       </c>
       <c r="G158" s="14" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H158" s="16" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I158" s="17" t="n">
         <v>18000</v>
@@ -8191,10 +8191,10 @@
         </is>
       </c>
       <c r="G159" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H159" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I159" s="13" t="n">
         <v>19000</v>
@@ -8238,10 +8238,10 @@
         </is>
       </c>
       <c r="G160" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H160" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I160" s="17" t="n">
         <v>8000</v>
@@ -8285,10 +8285,10 @@
         </is>
       </c>
       <c r="G161" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H161" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I161" s="13" t="n">
         <v>8000</v>
@@ -8379,10 +8379,10 @@
         </is>
       </c>
       <c r="G163" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H163" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I163" s="13" t="n">
         <v>8000</v>
@@ -8426,10 +8426,10 @@
         </is>
       </c>
       <c r="G164" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H164" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I164" s="17" t="n">
         <v>11000</v>
@@ -8520,10 +8520,10 @@
         </is>
       </c>
       <c r="G166" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H166" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I166" s="17" t="n">
         <v>8000</v>
@@ -8661,10 +8661,10 @@
         </is>
       </c>
       <c r="G169" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H169" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I169" s="13" t="n">
         <v>8000</v>
@@ -8708,10 +8708,10 @@
         </is>
       </c>
       <c r="G170" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H170" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I170" s="17" t="n">
         <v>8000</v>
@@ -8755,10 +8755,10 @@
         </is>
       </c>
       <c r="G171" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H171" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I171" s="13" t="n">
         <v>8000</v>
@@ -8800,10 +8800,10 @@
         </is>
       </c>
       <c r="G172" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H172" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I172" s="17" t="n">
         <v>8000</v>
@@ -8892,10 +8892,10 @@
         </is>
       </c>
       <c r="G174" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H174" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I174" s="17" t="n">
         <v>8000</v>
@@ -8939,10 +8939,10 @@
         </is>
       </c>
       <c r="G175" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H175" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I175" s="13" t="n">
         <v>8000</v>
@@ -8984,10 +8984,10 @@
         </is>
       </c>
       <c r="G176" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H176" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I176" s="17" t="n">
         <v>8000</v>
@@ -9031,10 +9031,10 @@
         </is>
       </c>
       <c r="G177" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H177" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I177" s="13" t="n">
         <v>6500</v>
@@ -9125,10 +9125,10 @@
         </is>
       </c>
       <c r="G179" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H179" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I179" s="13" t="n">
         <v>8000</v>
@@ -9172,10 +9172,10 @@
         </is>
       </c>
       <c r="G180" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H180" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I180" s="17" t="n">
         <v>8000</v>
@@ -9266,10 +9266,10 @@
         </is>
       </c>
       <c r="G182" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H182" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I182" s="17" t="n">
         <v>4000</v>
@@ -9407,10 +9407,10 @@
         </is>
       </c>
       <c r="G185" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H185" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I185" s="13" t="n">
         <v>8000</v>
@@ -9454,10 +9454,10 @@
         </is>
       </c>
       <c r="G186" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H186" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I186" s="17" t="n">
         <v>8000</v>
@@ -9548,10 +9548,10 @@
         </is>
       </c>
       <c r="G188" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H188" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I188" s="17" t="n">
         <v>8000</v>
@@ -9593,10 +9593,10 @@
         </is>
       </c>
       <c r="G189" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H189" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I189" s="13" t="n">
         <v>8000</v>
@@ -9687,10 +9687,10 @@
         </is>
       </c>
       <c r="G191" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H191" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I191" s="13" t="n">
         <v>8000</v>
@@ -9734,10 +9734,10 @@
         </is>
       </c>
       <c r="G192" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H192" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I192" s="17" t="n">
         <v>8000</v>
@@ -9781,10 +9781,10 @@
         </is>
       </c>
       <c r="G193" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H193" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I193" s="13" t="n">
         <v>16000</v>
@@ -9875,10 +9875,10 @@
         </is>
       </c>
       <c r="G195" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H195" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I195" s="13" t="n">
         <v>19000</v>
@@ -9922,10 +9922,10 @@
         </is>
       </c>
       <c r="G196" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H196" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I196" s="17" t="n">
         <v>8000</v>
@@ -10016,10 +10016,10 @@
         </is>
       </c>
       <c r="G198" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H198" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I198" s="17" t="n">
         <v>8000</v>
@@ -10061,10 +10061,10 @@
         </is>
       </c>
       <c r="G199" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H199" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I199" s="13" t="n">
         <v>7000</v>
@@ -10108,10 +10108,10 @@
         </is>
       </c>
       <c r="G200" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H200" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I200" s="17" t="n">
         <v>8000</v>
@@ -10155,10 +10155,10 @@
         </is>
       </c>
       <c r="G201" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H201" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I201" s="13" t="n">
         <v>8000</v>
@@ -10202,10 +10202,10 @@
         </is>
       </c>
       <c r="G202" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H202" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I202" s="17" t="n">
         <v>8000</v>
@@ -10249,10 +10249,10 @@
         </is>
       </c>
       <c r="G203" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H203" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I203" s="13" t="n">
         <v>8000</v>
@@ -10296,10 +10296,10 @@
         </is>
       </c>
       <c r="G204" s="14" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H204" s="16" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I204" s="17" t="n">
         <v>16000</v>
@@ -10433,10 +10433,10 @@
         </is>
       </c>
       <c r="G207" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H207" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I207" s="13" t="n">
         <v>6500</v>
@@ -10480,10 +10480,10 @@
         </is>
       </c>
       <c r="G208" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H208" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I208" s="17" t="n">
         <v>8000</v>
@@ -10527,10 +10527,10 @@
         </is>
       </c>
       <c r="G209" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H209" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I209" s="13" t="n">
         <v>8000</v>
@@ -10668,10 +10668,10 @@
         </is>
       </c>
       <c r="G212" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H212" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I212" s="17" t="n">
         <v>8000</v>
@@ -10715,10 +10715,10 @@
         </is>
       </c>
       <c r="G213" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H213" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I213" s="13" t="n">
         <v>8000</v>
@@ -10760,10 +10760,10 @@
         </is>
       </c>
       <c r="G214" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H214" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I214" s="17" t="n">
         <v>4000</v>
@@ -10807,10 +10807,10 @@
         </is>
       </c>
       <c r="G215" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H215" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I215" s="13" t="n">
         <v>19000</v>
@@ -10854,10 +10854,10 @@
         </is>
       </c>
       <c r="G216" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H216" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I216" s="17" t="n">
         <v>8000</v>
@@ -10901,10 +10901,10 @@
         </is>
       </c>
       <c r="G217" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H217" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I217" s="13" t="n">
         <v>8000</v>
@@ -10948,10 +10948,10 @@
         </is>
       </c>
       <c r="G218" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H218" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I218" s="17" t="n">
         <v>8000</v>
@@ -10995,10 +10995,10 @@
         </is>
       </c>
       <c r="G219" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H219" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I219" s="13" t="n">
         <v>8000</v>
@@ -11042,10 +11042,10 @@
         </is>
       </c>
       <c r="G220" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H220" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I220" s="17" t="n">
         <v>8000</v>
@@ -11089,10 +11089,10 @@
         </is>
       </c>
       <c r="G221" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H221" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I221" s="13" t="n">
         <v>16000</v>
@@ -11136,10 +11136,10 @@
         </is>
       </c>
       <c r="G222" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H222" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I222" s="17" t="n">
         <v>8000</v>
@@ -11183,10 +11183,10 @@
         </is>
       </c>
       <c r="G223" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H223" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I223" s="13" t="n">
         <v>8000</v>
@@ -11275,10 +11275,10 @@
         </is>
       </c>
       <c r="G225" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H225" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I225" s="13" t="n">
         <v>7000</v>
@@ -11322,10 +11322,10 @@
         </is>
       </c>
       <c r="G226" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H226" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I226" s="17" t="n">
         <v>8000</v>
@@ -11369,10 +11369,10 @@
         </is>
       </c>
       <c r="G227" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H227" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I227" s="13" t="n">
         <v>8000</v>
@@ -11414,10 +11414,10 @@
         </is>
       </c>
       <c r="G228" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H228" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I228" s="17" t="n">
         <v>8000</v>
@@ -11461,10 +11461,10 @@
         </is>
       </c>
       <c r="G229" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H229" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I229" s="13" t="n">
         <v>8000</v>
@@ -11508,10 +11508,10 @@
         </is>
       </c>
       <c r="G230" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H230" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I230" s="17" t="n">
         <v>8000</v>
@@ -11555,10 +11555,10 @@
         </is>
       </c>
       <c r="G231" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H231" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I231" s="13" t="n">
         <v>6500</v>
@@ -11602,10 +11602,10 @@
         </is>
       </c>
       <c r="G232" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H232" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I232" s="17" t="n">
         <v>8000</v>
@@ -11649,10 +11649,10 @@
         </is>
       </c>
       <c r="G233" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H233" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I233" s="13" t="n">
         <v>4000</v>
@@ -11696,10 +11696,10 @@
         </is>
       </c>
       <c r="G234" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H234" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I234" s="17" t="n">
         <v>8000</v>
@@ -11743,10 +11743,10 @@
         </is>
       </c>
       <c r="G235" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H235" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I235" s="13" t="n">
         <v>8000</v>
@@ -11790,10 +11790,10 @@
         </is>
       </c>
       <c r="G236" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H236" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I236" s="17" t="n">
         <v>6500</v>
@@ -11837,10 +11837,10 @@
         </is>
       </c>
       <c r="G237" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H237" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I237" s="13" t="n">
         <v>8000</v>
@@ -11884,10 +11884,10 @@
         </is>
       </c>
       <c r="G238" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H238" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I238" s="17" t="n">
         <v>8000</v>
@@ -11931,10 +11931,10 @@
         </is>
       </c>
       <c r="G239" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H239" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I239" s="13" t="n">
         <v>8000</v>
@@ -11978,10 +11978,10 @@
         </is>
       </c>
       <c r="G240" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H240" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I240" s="17" t="n">
         <v>4000</v>
@@ -12025,10 +12025,10 @@
         </is>
       </c>
       <c r="G241" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H241" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I241" s="13" t="n">
         <v>6500</v>
@@ -12072,10 +12072,10 @@
         </is>
       </c>
       <c r="G242" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H242" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I242" s="17" t="n">
         <v>8000</v>
@@ -12119,10 +12119,10 @@
         </is>
       </c>
       <c r="G243" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H243" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I243" s="13" t="n">
         <v>6500</v>
@@ -12166,10 +12166,10 @@
         </is>
       </c>
       <c r="G244" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H244" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I244" s="17" t="n">
         <v>8000</v>
@@ -12213,10 +12213,10 @@
         </is>
       </c>
       <c r="G245" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H245" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I245" s="13" t="n">
         <v>8000</v>
@@ -12260,10 +12260,10 @@
         </is>
       </c>
       <c r="G246" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H246" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I246" s="17" t="n">
         <v>4000</v>
@@ -12542,10 +12542,10 @@
         </is>
       </c>
       <c r="G252" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H252" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I252" s="17" t="n">
         <v>8000</v>
@@ -12589,10 +12589,10 @@
         </is>
       </c>
       <c r="G253" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H253" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I253" s="13" t="n">
         <v>8000</v>
@@ -12777,10 +12777,10 @@
         </is>
       </c>
       <c r="G257" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H257" s="6" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="I257" s="13" t="n">
         <v>16000</v>
@@ -12824,10 +12824,10 @@
         </is>
       </c>
       <c r="G258" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H258" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I258" s="17" t="n">
         <v>8000</v>
@@ -12871,10 +12871,10 @@
         </is>
       </c>
       <c r="G259" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H259" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I259" s="13" t="n">
         <v>8000</v>
@@ -12918,10 +12918,10 @@
         </is>
       </c>
       <c r="G260" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H260" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I260" s="17" t="n">
         <v>4000</v>
@@ -12965,10 +12965,10 @@
         </is>
       </c>
       <c r="G261" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H261" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I261" s="13" t="n">
         <v>8000</v>
@@ -13012,10 +13012,10 @@
         </is>
       </c>
       <c r="G262" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H262" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I262" s="17" t="n">
         <v>4000</v>
@@ -13059,10 +13059,10 @@
         </is>
       </c>
       <c r="G263" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H263" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I263" s="13" t="n">
         <v>7000</v>
@@ -13106,10 +13106,10 @@
         </is>
       </c>
       <c r="G264" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H264" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I264" s="17" t="n">
         <v>8000</v>
@@ -13151,10 +13151,10 @@
         </is>
       </c>
       <c r="G265" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H265" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I265" s="13" t="n">
         <v>8000</v>
@@ -13196,10 +13196,10 @@
         </is>
       </c>
       <c r="G266" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H266" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I266" s="17" t="n">
         <v>8000</v>
@@ -13241,10 +13241,10 @@
         </is>
       </c>
       <c r="G267" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H267" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I267" s="13" t="n">
         <v>8000</v>
@@ -13421,10 +13421,10 @@
         </is>
       </c>
       <c r="G271" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H271" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I271" s="13" t="n">
         <v>4000</v>
@@ -13511,10 +13511,10 @@
         </is>
       </c>
       <c r="G273" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H273" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I273" s="13" t="n">
         <v>8000</v>
@@ -13556,10 +13556,10 @@
         </is>
       </c>
       <c r="G274" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H274" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I274" s="17" t="n">
         <v>8000</v>
@@ -13601,10 +13601,10 @@
         </is>
       </c>
       <c r="G275" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H275" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I275" s="13" t="n">
         <v>8000</v>
@@ -13781,10 +13781,10 @@
         </is>
       </c>
       <c r="G279" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H279" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I279" s="13" t="n">
         <v>8000</v>
@@ -13826,10 +13826,10 @@
         </is>
       </c>
       <c r="G280" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H280" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I280" s="17" t="n">
         <v>7000</v>
@@ -13871,10 +13871,10 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H281" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I281" s="13" t="n">
         <v>4000</v>
@@ -13916,10 +13916,10 @@
         </is>
       </c>
       <c r="G282" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H282" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I282" s="17" t="n">
         <v>8000</v>
@@ -13961,10 +13961,10 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H283" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I283" s="13" t="n">
         <v>8000</v>
@@ -14051,10 +14051,10 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H285" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I285" s="13" t="n">
         <v>8000</v>
@@ -14096,10 +14096,10 @@
         </is>
       </c>
       <c r="G286" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H286" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I286" s="17" t="n">
         <v>8000</v>
@@ -14186,10 +14186,10 @@
         </is>
       </c>
       <c r="G288" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H288" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I288" s="17" t="n">
         <v>8000</v>
@@ -14231,10 +14231,10 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H289" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I289" s="13" t="n">
         <v>8000</v>
@@ -14276,10 +14276,10 @@
         </is>
       </c>
       <c r="G290" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H290" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I290" s="17" t="n">
         <v>8000</v>
@@ -14321,10 +14321,10 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H291" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I291" s="13" t="n">
         <v>8000</v>
@@ -14366,10 +14366,10 @@
         </is>
       </c>
       <c r="G292" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H292" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I292" s="17" t="n">
         <v>7000</v>
@@ -14411,10 +14411,10 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H293" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I293" s="13" t="n">
         <v>8000</v>
@@ -14591,10 +14591,10 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H297" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I297" s="13" t="n">
         <v>8000</v>
@@ -14636,10 +14636,10 @@
         </is>
       </c>
       <c r="G298" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H298" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I298" s="17" t="n">
         <v>8000</v>
@@ -14726,10 +14726,10 @@
         </is>
       </c>
       <c r="G300" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H300" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I300" s="17" t="n">
         <v>8000</v>
@@ -14771,10 +14771,10 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H301" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I301" s="13" t="n">
         <v>8000</v>
@@ -14816,10 +14816,10 @@
         </is>
       </c>
       <c r="G302" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H302" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I302" s="17" t="n">
         <v>8000</v>
@@ -14861,10 +14861,10 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H303" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I303" s="13" t="n">
         <v>8000</v>
@@ -14906,10 +14906,10 @@
         </is>
       </c>
       <c r="G304" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H304" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I304" s="17" t="n">
         <v>8000</v>
@@ -14996,10 +14996,10 @@
         </is>
       </c>
       <c r="G306" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H306" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I306" s="17" t="n">
         <v>8000</v>
@@ -15041,10 +15041,10 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H307" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I307" s="13" t="n">
         <v>8000</v>
@@ -15086,10 +15086,10 @@
         </is>
       </c>
       <c r="G308" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H308" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I308" s="17" t="n">
         <v>8000</v>
@@ -15131,10 +15131,10 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H309" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I309" s="13" t="n">
         <v>8000</v>
@@ -15176,10 +15176,10 @@
         </is>
       </c>
       <c r="G310" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H310" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I310" s="17" t="n">
         <v>8000</v>
@@ -15221,10 +15221,10 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H311" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I311" s="13" t="n">
         <v>8000</v>
@@ -15266,10 +15266,10 @@
         </is>
       </c>
       <c r="G312" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H312" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I312" s="17" t="n">
         <v>8000</v>
@@ -15311,10 +15311,10 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H313" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I313" s="13" t="n">
         <v>8000</v>
@@ -15356,10 +15356,10 @@
         </is>
       </c>
       <c r="G314" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H314" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I314" s="17" t="n">
         <v>8000</v>
@@ -15401,10 +15401,10 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H315" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I315" s="13" t="n">
         <v>8000</v>
@@ -15446,10 +15446,10 @@
         </is>
       </c>
       <c r="G316" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H316" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I316" s="17" t="n">
         <v>8000</v>
@@ -15491,10 +15491,10 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H317" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I317" s="13" t="n">
         <v>4000</v>
@@ -15536,10 +15536,10 @@
         </is>
       </c>
       <c r="G318" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H318" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I318" s="17" t="n">
         <v>8000</v>
@@ -15581,10 +15581,10 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H319" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I319" s="13" t="n">
         <v>8000</v>
@@ -15626,10 +15626,10 @@
         </is>
       </c>
       <c r="G320" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H320" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I320" s="17" t="n">
         <v>8000</v>
@@ -15671,10 +15671,10 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H321" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I321" s="13" t="n">
         <v>8000</v>
@@ -15758,13 +15758,13 @@
         <v>105</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>17800000</v>
+        <v>13911000</v>
       </c>
       <c r="D3" t="n">
         <v>32.9</v>
       </c>
       <c r="E3" t="n">
-        <v>31.8</v>
+        <v>30.8</v>
       </c>
     </row>
     <row r="4">
@@ -15777,13 +15777,13 @@
         <v>47</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>9700000</v>
+        <v>8573000</v>
       </c>
       <c r="D4" t="n">
         <v>14.7</v>
       </c>
       <c r="E4" t="n">
-        <v>17.3</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -15796,13 +15796,13 @@
         <v>35</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>6850000</v>
+        <v>5573000</v>
       </c>
       <c r="D5" t="n">
         <v>11</v>
       </c>
       <c r="E5" t="n">
-        <v>12.2</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="6">
@@ -15815,13 +15815,13 @@
         <v>59</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>9600000</v>
+        <v>7219000</v>
       </c>
       <c r="D6" t="n">
         <v>18.5</v>
       </c>
       <c r="E6" t="n">
-        <v>17.1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -15834,13 +15834,13 @@
         <v>61</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>10350000</v>
+        <v>8600000</v>
       </c>
       <c r="D7" t="n">
         <v>19.1</v>
       </c>
       <c r="E7" t="n">
-        <v>18.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8">
@@ -15853,13 +15853,13 @@
         <v>12</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1723000</v>
+        <v>1273000</v>
       </c>
       <c r="D8" t="n">
         <v>3.8</v>
       </c>
       <c r="E8" t="n">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="9">
@@ -15872,7 +15872,7 @@
         <v>319</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>56023000</v>
+        <v>45149000</v>
       </c>
     </row>
   </sheetData>
@@ -15935,16 +15935,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C3" s="6" t="n">
         <v>73000</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>73000</v>
+        <v>949000</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="4">
@@ -15952,16 +15952,16 @@
         <v>12</v>
       </c>
       <c r="B4" t="n">
-        <v>29</v>
+        <v>182</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>100000</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>2900000</v>
+        <v>18200000</v>
       </c>
       <c r="E4" t="n">
-        <v>9.1</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="5">
@@ -15969,16 +15969,16 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>181</v>
+        <v>31</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>150000</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>27150000</v>
+        <v>4650000</v>
       </c>
       <c r="E5" t="n">
-        <v>56.7</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -15986,16 +15986,16 @@
         <v>30</v>
       </c>
       <c r="B6" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>200000</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>4400000</v>
+        <v>7600000</v>
       </c>
       <c r="E6" t="n">
-        <v>6.9</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="7">
@@ -16003,16 +16003,16 @@
         <v>50</v>
       </c>
       <c r="B7" t="n">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>250000</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>21500000</v>
+        <v>13750000</v>
       </c>
       <c r="E7" t="n">
-        <v>27</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="8">
@@ -16025,7 +16025,7 @@
         <v>319</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>56023000</v>
+        <v>45149000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simplify to 3 capacity tiers with 30/30/40 rank-based distribution
- shelter_capacity.py: assign tiers by traffic rank (bottom 30%→6p,
  next 30%→12p, top 40%→20p); removes threshold-based rounding
- export_final_placements.py: drop alert upgrade logic; tiers are
  set by rank in shelter_capacity.py, just pass through
- shelter_capacity_map.py: remove upgrade annotations; 3 tiers only
- create_budget_excel_v2.py: 3 tiers only (6/12/20p)
- Result: 96×6p / 95×12p / 128×20p; capital ₪35.7M, 10-yr ₪88.9M

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/budget_shelters_v2.xlsx
+++ b/budget_shelters_v2.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -558,7 +558,7 @@
         <v>73000</v>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>96</v>
       </c>
       <c r="D6" s="6">
         <f>B6*C6</f>
@@ -573,7 +573,7 @@
         <v>100000</v>
       </c>
       <c r="C7" t="n">
-        <v>182</v>
+        <v>95</v>
       </c>
       <c r="D7" s="6">
         <f>B7*C7</f>
@@ -588,7 +588,7 @@
         <v>150000</v>
       </c>
       <c r="C8" t="n">
-        <v>31</v>
+        <v>128</v>
       </c>
       <c r="D8" s="6">
         <f>B8*C8</f>
@@ -596,147 +596,117 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>30</v>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>200000</v>
-      </c>
-      <c r="C9" t="n">
-        <v>38</v>
-      </c>
-      <c r="D9" s="6">
-        <f>B9*C9</f>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>עלות הון סה"כ</t>
+        </is>
+      </c>
+      <c r="D9" s="7">
+        <f>D6+D7+D8</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>50</v>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>250000</v>
-      </c>
-      <c r="C10" t="n">
-        <v>55</v>
-      </c>
-      <c r="D10" s="6">
-        <f>B10*C10</f>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>פרמטרים נוספים (ניתן לשינוי)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>רזרבה / אי-וודאות (%)</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>עלות תחזוקה שנתית לכל מיגונית (₪)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>סיכום תקציבי</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>מספר מיגוניות</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>עלות הון (ללא מע"מ)</t>
+        </is>
+      </c>
+      <c r="B17" s="6">
+        <f>D9</f>
         <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>עלות הון סה"כ</t>
-        </is>
-      </c>
-      <c r="D11" s="7">
-        <f>D6+D7+D8+D9+D10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>פרמטרים נוספים (ניתן לשינוי)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>רזרבה / אי-וודאות (%)</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>עלות תחזוקה שנתית לכל מיגונית (₪)</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>סיכום תקציבי</t>
-        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>מספר מיגוניות</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>319</v>
+          <t>רזרבה</t>
+        </is>
+      </c>
+      <c r="B18" s="6">
+        <f>D9*B12/100</f>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>עלות הון (ללא מע"מ)</t>
-        </is>
-      </c>
-      <c r="B19" s="6">
-        <f>D11</f>
+          <t>עלות הון כולל רזרבה</t>
+        </is>
+      </c>
+      <c r="B19" s="7">
+        <f>D9*(1+B12/100)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>רזרבה</t>
+          <t>עלות תחזוקה שנתית (319 מיגוניות)</t>
         </is>
       </c>
       <c r="B20" s="6">
-        <f>D11*B14/100</f>
+        <f>B13*319</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>עלות הון כולל רזרבה</t>
+          <t>עלות כוללת ל-10 שנים</t>
         </is>
       </c>
       <c r="B21" s="7">
-        <f>D11*(1+B14/100)</f>
+        <f>D9*(1+B12/100)+B13*319*10</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>עלות תחזוקה שנתית (319 מיגוניות)</t>
-        </is>
-      </c>
-      <c r="B22" s="6">
-        <f>B15*319</f>
-        <v/>
-      </c>
-    </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>עלות כוללת ל-10 שנים</t>
-        </is>
-      </c>
-      <c r="B23" s="7">
-        <f>D11*(1+B14/100)+B15*319*10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>הערות: עלויות ללא מע"מ. מבוסס על אלגוריתם Gonzalez k-center | תקן 5 דקות | 319 מיגוניות | ישראל בלבד (קו ירוק 1967) | קיבולת מחושבת לפי תנועה בשעת שיא בזמן מלחמה (10% מתנועה רגילה)</t>
         </is>
@@ -875,10 +845,10 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I3" s="13" t="n">
         <v>8000</v>
@@ -922,10 +892,10 @@
         </is>
       </c>
       <c r="G4" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H4" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I4" s="17" t="n">
         <v>9000</v>
@@ -969,10 +939,10 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I5" s="13" t="n">
         <v>20000</v>
@@ -1016,10 +986,10 @@
         </is>
       </c>
       <c r="G6" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I6" s="17" t="n">
         <v>20000</v>
@@ -1110,10 +1080,10 @@
         </is>
       </c>
       <c r="G8" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I8" s="17" t="n">
         <v>18000</v>
@@ -1157,10 +1127,10 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>150000</v>
+        <v>73000</v>
       </c>
       <c r="I9" s="13" t="n">
         <v>4000</v>
@@ -1204,10 +1174,10 @@
         </is>
       </c>
       <c r="G10" s="14" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I10" s="17" t="n">
         <v>8000</v>
@@ -1251,10 +1221,10 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I11" s="13" t="n">
         <v>9000</v>
@@ -1298,10 +1268,10 @@
         </is>
       </c>
       <c r="G12" s="14" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>150000</v>
+        <v>73000</v>
       </c>
       <c r="I12" s="17" t="n">
         <v>8000</v>
@@ -1345,10 +1315,10 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I13" s="13" t="n">
         <v>8000</v>
@@ -1392,10 +1362,10 @@
         </is>
       </c>
       <c r="G14" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I14" s="17" t="n">
         <v>7000</v>
@@ -1439,10 +1409,10 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I15" s="13" t="n">
         <v>30000</v>
@@ -1486,10 +1456,10 @@
         </is>
       </c>
       <c r="G16" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I16" s="17" t="n">
         <v>8000</v>
@@ -1533,10 +1503,10 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I17" s="13" t="n">
         <v>40000</v>
@@ -1580,10 +1550,10 @@
         </is>
       </c>
       <c r="G18" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H18" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I18" s="17" t="n">
         <v>18000</v>
@@ -1627,10 +1597,10 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I19" s="13" t="n">
         <v>8000</v>
@@ -1674,10 +1644,10 @@
         </is>
       </c>
       <c r="G20" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H20" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I20" s="17" t="n">
         <v>13000</v>
@@ -1721,10 +1691,10 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I21" s="13" t="n">
         <v>8000</v>
@@ -1768,10 +1738,10 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H22" s="16" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I22" s="17" t="n">
         <v>8000</v>
@@ -1815,10 +1785,10 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I23" s="13" t="n">
         <v>8000</v>
@@ -1862,10 +1832,10 @@
         </is>
       </c>
       <c r="G24" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H24" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I24" s="17" t="n">
         <v>40000</v>
@@ -1909,10 +1879,10 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I25" s="13" t="n">
         <v>8000</v>
@@ -1956,10 +1926,10 @@
         </is>
       </c>
       <c r="G26" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H26" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I26" s="17" t="n">
         <v>8000</v>
@@ -2003,10 +1973,10 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I27" s="13" t="n">
         <v>8000</v>
@@ -2050,10 +2020,10 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H28" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I28" s="17" t="n">
         <v>40000</v>
@@ -2097,10 +2067,10 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I29" s="13" t="n">
         <v>8000</v>
@@ -2144,10 +2114,10 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H30" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I30" s="17" t="n">
         <v>40000</v>
@@ -2191,10 +2161,10 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I31" s="13" t="n">
         <v>40000</v>
@@ -2238,10 +2208,10 @@
         </is>
       </c>
       <c r="G32" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H32" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I32" s="17" t="n">
         <v>7000</v>
@@ -2285,10 +2255,10 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I33" s="13" t="n">
         <v>8000</v>
@@ -2332,10 +2302,10 @@
         </is>
       </c>
       <c r="G34" s="14" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H34" s="16" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I34" s="17" t="n">
         <v>8000</v>
@@ -2379,10 +2349,10 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I35" s="13" t="n">
         <v>8000</v>
@@ -2426,10 +2396,10 @@
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H36" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I36" s="17" t="n">
         <v>30000</v>
@@ -2473,10 +2443,10 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I37" s="13" t="n">
         <v>7000</v>
@@ -2518,10 +2488,10 @@
         </is>
       </c>
       <c r="G38" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H38" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I38" s="17" t="n">
         <v>13000</v>
@@ -2565,10 +2535,10 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I39" s="13" t="n">
         <v>13000</v>
@@ -2612,10 +2582,10 @@
         </is>
       </c>
       <c r="G40" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H40" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I40" s="17" t="n">
         <v>20000</v>
@@ -2659,10 +2629,10 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I41" s="13" t="n">
         <v>8000</v>
@@ -2706,10 +2676,10 @@
         </is>
       </c>
       <c r="G42" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H42" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I42" s="17" t="n">
         <v>30000</v>
@@ -2753,10 +2723,10 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I43" s="13" t="n">
         <v>40000</v>
@@ -2800,10 +2770,10 @@
         </is>
       </c>
       <c r="G44" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H44" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I44" s="17" t="n">
         <v>8000</v>
@@ -2847,10 +2817,10 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I45" s="13" t="n">
         <v>8000</v>
@@ -2894,10 +2864,10 @@
         </is>
       </c>
       <c r="G46" s="14" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H46" s="16" t="n">
-        <v>150000</v>
+        <v>73000</v>
       </c>
       <c r="I46" s="17" t="n">
         <v>8000</v>
@@ -2941,10 +2911,10 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>150000</v>
+        <v>73000</v>
       </c>
       <c r="I47" s="13" t="n">
         <v>8000</v>
@@ -2988,10 +2958,10 @@
         </is>
       </c>
       <c r="G48" s="14" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H48" s="16" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I48" s="17" t="n">
         <v>8000</v>
@@ -3035,10 +3005,10 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I49" s="13" t="n">
         <v>8000</v>
@@ -3082,10 +3052,10 @@
         </is>
       </c>
       <c r="G50" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H50" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I50" s="17" t="n">
         <v>9000</v>
@@ -3129,10 +3099,10 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H51" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I51" s="13" t="n">
         <v>7000</v>
@@ -3176,10 +3146,10 @@
         </is>
       </c>
       <c r="G52" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H52" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I52" s="17" t="n">
         <v>8500</v>
@@ -3223,10 +3193,10 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H53" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I53" s="13" t="n">
         <v>9000</v>
@@ -3270,10 +3240,10 @@
         </is>
       </c>
       <c r="G54" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H54" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I54" s="17" t="n">
         <v>15000</v>
@@ -3317,10 +3287,10 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H55" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I55" s="13" t="n">
         <v>20000</v>
@@ -3364,10 +3334,10 @@
         </is>
       </c>
       <c r="G56" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H56" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I56" s="17" t="n">
         <v>18000</v>
@@ -3411,10 +3381,10 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H57" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I57" s="13" t="n">
         <v>8500</v>
@@ -3458,10 +3428,10 @@
         </is>
       </c>
       <c r="G58" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H58" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I58" s="17" t="n">
         <v>8000</v>
@@ -3505,10 +3475,10 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H59" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I59" s="13" t="n">
         <v>8000</v>
@@ -3550,10 +3520,10 @@
         </is>
       </c>
       <c r="G60" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H60" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I60" s="17" t="n">
         <v>7000</v>
@@ -3597,10 +3567,10 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H61" s="6" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I61" s="13" t="n">
         <v>8000</v>
@@ -3644,10 +3614,10 @@
         </is>
       </c>
       <c r="G62" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H62" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I62" s="17" t="n">
         <v>9000</v>
@@ -3738,10 +3708,10 @@
         </is>
       </c>
       <c r="G64" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H64" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I64" s="17" t="n">
         <v>7000</v>
@@ -3832,10 +3802,10 @@
         </is>
       </c>
       <c r="G66" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H66" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I66" s="17" t="n">
         <v>7000</v>
@@ -3877,10 +3847,10 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H67" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I67" s="13" t="n">
         <v>8000</v>
@@ -3924,10 +3894,10 @@
         </is>
       </c>
       <c r="G68" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H68" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I68" s="17" t="n">
         <v>8000</v>
@@ -3971,10 +3941,10 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H69" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I69" s="13" t="n">
         <v>8000</v>
@@ -4018,10 +3988,10 @@
         </is>
       </c>
       <c r="G70" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H70" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I70" s="17" t="n">
         <v>30000</v>
@@ -4065,10 +4035,10 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H71" s="6" t="n">
-        <v>200000</v>
+        <v>73000</v>
       </c>
       <c r="I71" s="13" t="n">
         <v>8000</v>
@@ -4112,10 +4082,10 @@
         </is>
       </c>
       <c r="G72" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H72" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I72" s="17" t="n">
         <v>8000</v>
@@ -4157,10 +4127,10 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H73" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I73" s="13" t="n">
         <v>40000</v>
@@ -4204,10 +4174,10 @@
         </is>
       </c>
       <c r="G74" s="14" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H74" s="16" t="n">
-        <v>150000</v>
+        <v>73000</v>
       </c>
       <c r="I74" s="17" t="n">
         <v>8000</v>
@@ -4251,10 +4221,10 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H75" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I75" s="13" t="n">
         <v>4000</v>
@@ -4345,10 +4315,10 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H77" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I77" s="13" t="n">
         <v>8000</v>
@@ -4392,10 +4362,10 @@
         </is>
       </c>
       <c r="G78" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H78" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I78" s="17" t="n">
         <v>18000</v>
@@ -4439,10 +4409,10 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H79" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I79" s="13" t="n">
         <v>20000</v>
@@ -4486,10 +4456,10 @@
         </is>
       </c>
       <c r="G80" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H80" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I80" s="17" t="n">
         <v>8000</v>
@@ -4533,10 +4503,10 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H81" s="6" t="n">
-        <v>150000</v>
+        <v>73000</v>
       </c>
       <c r="I81" s="13" t="n">
         <v>8000</v>
@@ -4580,10 +4550,10 @@
         </is>
       </c>
       <c r="G82" s="14" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H82" s="16" t="n">
-        <v>150000</v>
+        <v>73000</v>
       </c>
       <c r="I82" s="17" t="n">
         <v>8000</v>
@@ -4627,10 +4597,10 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H83" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I83" s="13" t="n">
         <v>8000</v>
@@ -4674,10 +4644,10 @@
         </is>
       </c>
       <c r="G84" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H84" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I84" s="17" t="n">
         <v>18000</v>
@@ -4721,10 +4691,10 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H85" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I85" s="13" t="n">
         <v>7000</v>
@@ -4766,10 +4736,10 @@
         </is>
       </c>
       <c r="G86" s="14" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H86" s="16" t="n">
-        <v>150000</v>
+        <v>73000</v>
       </c>
       <c r="I86" s="17" t="n">
         <v>8000</v>
@@ -4813,10 +4783,10 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H87" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I87" s="13" t="n">
         <v>8000</v>
@@ -4860,10 +4830,10 @@
         </is>
       </c>
       <c r="G88" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H88" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I88" s="17" t="n">
         <v>4000</v>
@@ -4954,10 +4924,10 @@
         </is>
       </c>
       <c r="G90" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H90" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I90" s="17" t="n">
         <v>22000</v>
@@ -5001,10 +4971,10 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H91" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I91" s="13" t="n">
         <v>8000</v>
@@ -5048,10 +5018,10 @@
         </is>
       </c>
       <c r="G92" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H92" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I92" s="17" t="n">
         <v>8000</v>
@@ -5095,10 +5065,10 @@
         </is>
       </c>
       <c r="G93" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H93" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I93" s="13" t="n">
         <v>13000</v>
@@ -5142,10 +5112,10 @@
         </is>
       </c>
       <c r="G94" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H94" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I94" s="17" t="n">
         <v>18000</v>
@@ -5189,10 +5159,10 @@
         </is>
       </c>
       <c r="G95" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H95" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I95" s="13" t="n">
         <v>8000</v>
@@ -5236,10 +5206,10 @@
         </is>
       </c>
       <c r="G96" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H96" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I96" s="17" t="n">
         <v>4000</v>
@@ -5283,10 +5253,10 @@
         </is>
       </c>
       <c r="G97" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H97" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I97" s="13" t="n">
         <v>8000</v>
@@ -5377,10 +5347,10 @@
         </is>
       </c>
       <c r="G99" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H99" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I99" s="13" t="n">
         <v>8000</v>
@@ -5424,10 +5394,10 @@
         </is>
       </c>
       <c r="G100" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H100" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I100" s="17" t="n">
         <v>8000</v>
@@ -5471,10 +5441,10 @@
         </is>
       </c>
       <c r="G101" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H101" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I101" s="13" t="n">
         <v>13000</v>
@@ -5518,10 +5488,10 @@
         </is>
       </c>
       <c r="G102" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H102" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I102" s="17" t="n">
         <v>14000</v>
@@ -5565,10 +5535,10 @@
         </is>
       </c>
       <c r="G103" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H103" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I103" s="13" t="n">
         <v>8000</v>
@@ -5704,10 +5674,10 @@
         </is>
       </c>
       <c r="G106" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H106" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I106" s="17" t="n">
         <v>22000</v>
@@ -5798,10 +5768,10 @@
         </is>
       </c>
       <c r="G108" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H108" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I108" s="17" t="n">
         <v>35000</v>
@@ -5890,10 +5860,10 @@
         </is>
       </c>
       <c r="G110" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H110" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I110" s="17" t="n">
         <v>4000</v>
@@ -6031,10 +6001,10 @@
         </is>
       </c>
       <c r="G113" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H113" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I113" s="13" t="n">
         <v>13000</v>
@@ -6078,10 +6048,10 @@
         </is>
       </c>
       <c r="G114" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H114" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I114" s="17" t="n">
         <v>8000</v>
@@ -6266,10 +6236,10 @@
         </is>
       </c>
       <c r="G118" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H118" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I118" s="17" t="n">
         <v>8000</v>
@@ -6454,10 +6424,10 @@
         </is>
       </c>
       <c r="G122" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H122" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I122" s="17" t="n">
         <v>7000</v>
@@ -6548,10 +6518,10 @@
         </is>
       </c>
       <c r="G124" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H124" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I124" s="17" t="n">
         <v>8000</v>
@@ -6783,10 +6753,10 @@
         </is>
       </c>
       <c r="G129" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H129" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I129" s="13" t="n">
         <v>4000</v>
@@ -6971,10 +6941,10 @@
         </is>
       </c>
       <c r="G133" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H133" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I133" s="13" t="n">
         <v>24000</v>
@@ -7065,10 +7035,10 @@
         </is>
       </c>
       <c r="G135" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H135" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I135" s="13" t="n">
         <v>22000</v>
@@ -7253,10 +7223,10 @@
         </is>
       </c>
       <c r="G139" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H139" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I139" s="13" t="n">
         <v>20000</v>
@@ -7300,10 +7270,10 @@
         </is>
       </c>
       <c r="G140" s="14" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H140" s="16" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I140" s="17" t="n">
         <v>8000</v>
@@ -7394,10 +7364,10 @@
         </is>
       </c>
       <c r="G142" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H142" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I142" s="17" t="n">
         <v>18000</v>
@@ -7629,10 +7599,10 @@
         </is>
       </c>
       <c r="G147" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H147" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I147" s="13" t="n">
         <v>19000</v>
@@ -7676,10 +7646,10 @@
         </is>
       </c>
       <c r="G148" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H148" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I148" s="17" t="n">
         <v>22000</v>
@@ -7770,10 +7740,10 @@
         </is>
       </c>
       <c r="G150" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H150" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I150" s="17" t="n">
         <v>24000</v>
@@ -7862,10 +7832,10 @@
         </is>
       </c>
       <c r="G152" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H152" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I152" s="17" t="n">
         <v>13000</v>
@@ -7956,10 +7926,10 @@
         </is>
       </c>
       <c r="G154" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H154" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I154" s="17" t="n">
         <v>13000</v>
@@ -8050,10 +8020,10 @@
         </is>
       </c>
       <c r="G156" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H156" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I156" s="17" t="n">
         <v>24000</v>
@@ -8144,10 +8114,10 @@
         </is>
       </c>
       <c r="G158" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H158" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I158" s="17" t="n">
         <v>18000</v>
@@ -8191,10 +8161,10 @@
         </is>
       </c>
       <c r="G159" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H159" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I159" s="13" t="n">
         <v>19000</v>
@@ -8332,10 +8302,10 @@
         </is>
       </c>
       <c r="G162" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H162" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I162" s="17" t="n">
         <v>4000</v>
@@ -8473,10 +8443,10 @@
         </is>
       </c>
       <c r="G165" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H165" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I165" s="13" t="n">
         <v>22000</v>
@@ -8567,10 +8537,10 @@
         </is>
       </c>
       <c r="G167" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H167" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I167" s="13" t="n">
         <v>24000</v>
@@ -8614,10 +8584,10 @@
         </is>
       </c>
       <c r="G168" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H168" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I168" s="17" t="n">
         <v>22000</v>
@@ -9031,10 +9001,10 @@
         </is>
       </c>
       <c r="G177" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H177" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I177" s="13" t="n">
         <v>6500</v>
@@ -9078,10 +9048,10 @@
         </is>
       </c>
       <c r="G178" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H178" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I178" s="17" t="n">
         <v>4000</v>
@@ -9219,10 +9189,10 @@
         </is>
       </c>
       <c r="G181" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H181" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I181" s="13" t="n">
         <v>14000</v>
@@ -9360,10 +9330,10 @@
         </is>
       </c>
       <c r="G184" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H184" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I184" s="17" t="n">
         <v>4000</v>
@@ -9501,10 +9471,10 @@
         </is>
       </c>
       <c r="G187" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H187" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I187" s="13" t="n">
         <v>22000</v>
@@ -9640,10 +9610,10 @@
         </is>
       </c>
       <c r="G190" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H190" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I190" s="17" t="n">
         <v>4000</v>
@@ -9781,10 +9751,10 @@
         </is>
       </c>
       <c r="G193" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H193" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I193" s="13" t="n">
         <v>16000</v>
@@ -9828,10 +9798,10 @@
         </is>
       </c>
       <c r="G194" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H194" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I194" s="17" t="n">
         <v>13000</v>
@@ -9875,10 +9845,10 @@
         </is>
       </c>
       <c r="G195" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H195" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I195" s="13" t="n">
         <v>19000</v>
@@ -9969,10 +9939,10 @@
         </is>
       </c>
       <c r="G197" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H197" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I197" s="13" t="n">
         <v>13000</v>
@@ -10061,10 +10031,10 @@
         </is>
       </c>
       <c r="G199" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H199" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I199" s="13" t="n">
         <v>7000</v>
@@ -10296,10 +10266,10 @@
         </is>
       </c>
       <c r="G204" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H204" s="16" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I204" s="17" t="n">
         <v>16000</v>
@@ -10343,10 +10313,10 @@
         </is>
       </c>
       <c r="G205" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H205" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I205" s="13" t="n">
         <v>22000</v>
@@ -10388,10 +10358,10 @@
         </is>
       </c>
       <c r="G206" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H206" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I206" s="17" t="n">
         <v>22000</v>
@@ -10433,10 +10403,10 @@
         </is>
       </c>
       <c r="G207" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H207" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I207" s="13" t="n">
         <v>6500</v>
@@ -10574,10 +10544,10 @@
         </is>
       </c>
       <c r="G210" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H210" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I210" s="17" t="n">
         <v>24000</v>
@@ -10621,10 +10591,10 @@
         </is>
       </c>
       <c r="G211" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H211" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I211" s="13" t="n">
         <v>24000</v>
@@ -10807,10 +10777,10 @@
         </is>
       </c>
       <c r="G215" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H215" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I215" s="13" t="n">
         <v>19000</v>
@@ -11089,10 +11059,10 @@
         </is>
       </c>
       <c r="G221" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H221" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I221" s="13" t="n">
         <v>16000</v>
@@ -11230,10 +11200,10 @@
         </is>
       </c>
       <c r="G224" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H224" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I224" s="17" t="n">
         <v>22000</v>
@@ -11275,10 +11245,10 @@
         </is>
       </c>
       <c r="G225" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H225" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I225" s="13" t="n">
         <v>7000</v>
@@ -11555,10 +11525,10 @@
         </is>
       </c>
       <c r="G231" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H231" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I231" s="13" t="n">
         <v>6500</v>
@@ -11790,10 +11760,10 @@
         </is>
       </c>
       <c r="G236" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H236" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I236" s="17" t="n">
         <v>6500</v>
@@ -12025,10 +11995,10 @@
         </is>
       </c>
       <c r="G241" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H241" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I241" s="13" t="n">
         <v>6500</v>
@@ -12119,10 +12089,10 @@
         </is>
       </c>
       <c r="G243" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H243" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I243" s="13" t="n">
         <v>6500</v>
@@ -12307,10 +12277,10 @@
         </is>
       </c>
       <c r="G247" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H247" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I247" s="13" t="n">
         <v>22000</v>
@@ -12354,10 +12324,10 @@
         </is>
       </c>
       <c r="G248" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H248" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I248" s="17" t="n">
         <v>22000</v>
@@ -12401,10 +12371,10 @@
         </is>
       </c>
       <c r="G249" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H249" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I249" s="13" t="n">
         <v>22000</v>
@@ -12448,10 +12418,10 @@
         </is>
       </c>
       <c r="G250" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H250" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I250" s="17" t="n">
         <v>22000</v>
@@ -12495,10 +12465,10 @@
         </is>
       </c>
       <c r="G251" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H251" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I251" s="13" t="n">
         <v>22000</v>
@@ -12683,10 +12653,10 @@
         </is>
       </c>
       <c r="G255" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H255" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I255" s="13" t="n">
         <v>24000</v>
@@ -12730,10 +12700,10 @@
         </is>
       </c>
       <c r="G256" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H256" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I256" s="17" t="n">
         <v>24000</v>
@@ -12777,10 +12747,10 @@
         </is>
       </c>
       <c r="G257" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H257" s="6" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I257" s="13" t="n">
         <v>16000</v>
@@ -13059,10 +13029,10 @@
         </is>
       </c>
       <c r="G263" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H263" s="6" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I263" s="13" t="n">
         <v>7000</v>
@@ -13646,10 +13616,10 @@
         </is>
       </c>
       <c r="G276" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H276" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I276" s="17" t="n">
         <v>22000</v>
@@ -13691,10 +13661,10 @@
         </is>
       </c>
       <c r="G277" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H277" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I277" s="13" t="n">
         <v>22000</v>
@@ -13736,10 +13706,10 @@
         </is>
       </c>
       <c r="G278" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H278" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I278" s="17" t="n">
         <v>22000</v>
@@ -13826,10 +13796,10 @@
         </is>
       </c>
       <c r="G280" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H280" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I280" s="17" t="n">
         <v>7000</v>
@@ -13961,10 +13931,10 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H283" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I283" s="13" t="n">
         <v>8000</v>
@@ -14006,10 +13976,10 @@
         </is>
       </c>
       <c r="G284" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H284" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I284" s="17" t="n">
         <v>24000</v>
@@ -14051,10 +14021,10 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H285" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I285" s="13" t="n">
         <v>8000</v>
@@ -14096,10 +14066,10 @@
         </is>
       </c>
       <c r="G286" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H286" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I286" s="17" t="n">
         <v>8000</v>
@@ -14141,10 +14111,10 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H287" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I287" s="13" t="n">
         <v>22000</v>
@@ -14186,10 +14156,10 @@
         </is>
       </c>
       <c r="G288" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H288" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I288" s="17" t="n">
         <v>8000</v>
@@ -14231,10 +14201,10 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H289" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I289" s="13" t="n">
         <v>8000</v>
@@ -14276,10 +14246,10 @@
         </is>
       </c>
       <c r="G290" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H290" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I290" s="17" t="n">
         <v>8000</v>
@@ -14321,10 +14291,10 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H291" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I291" s="13" t="n">
         <v>8000</v>
@@ -14366,10 +14336,10 @@
         </is>
       </c>
       <c r="G292" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H292" s="16" t="n">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="I292" s="17" t="n">
         <v>7000</v>
@@ -14411,10 +14381,10 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H293" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I293" s="13" t="n">
         <v>8000</v>
@@ -14456,10 +14426,10 @@
         </is>
       </c>
       <c r="G294" s="14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H294" s="16" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I294" s="17" t="n">
         <v>22000</v>
@@ -14501,10 +14471,10 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H295" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I295" s="13" t="n">
         <v>22000</v>
@@ -14591,10 +14561,10 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H297" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I297" s="13" t="n">
         <v>8000</v>
@@ -14636,10 +14606,10 @@
         </is>
       </c>
       <c r="G298" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H298" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I298" s="17" t="n">
         <v>8000</v>
@@ -14681,10 +14651,10 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H299" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I299" s="13" t="n">
         <v>22000</v>
@@ -14726,10 +14696,10 @@
         </is>
       </c>
       <c r="G300" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H300" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I300" s="17" t="n">
         <v>8000</v>
@@ -14771,10 +14741,10 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H301" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I301" s="13" t="n">
         <v>8000</v>
@@ -14816,10 +14786,10 @@
         </is>
       </c>
       <c r="G302" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H302" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I302" s="17" t="n">
         <v>8000</v>
@@ -14861,10 +14831,10 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H303" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I303" s="13" t="n">
         <v>8000</v>
@@ -14906,10 +14876,10 @@
         </is>
       </c>
       <c r="G304" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H304" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I304" s="17" t="n">
         <v>8000</v>
@@ -14951,10 +14921,10 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H305" s="6" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="I305" s="13" t="n">
         <v>24000</v>
@@ -14996,10 +14966,10 @@
         </is>
       </c>
       <c r="G306" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H306" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I306" s="17" t="n">
         <v>8000</v>
@@ -15041,10 +15011,10 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H307" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I307" s="13" t="n">
         <v>8000</v>
@@ -15086,10 +15056,10 @@
         </is>
       </c>
       <c r="G308" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H308" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I308" s="17" t="n">
         <v>8000</v>
@@ -15131,10 +15101,10 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H309" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I309" s="13" t="n">
         <v>8000</v>
@@ -15176,10 +15146,10 @@
         </is>
       </c>
       <c r="G310" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H310" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I310" s="17" t="n">
         <v>8000</v>
@@ -15221,10 +15191,10 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H311" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I311" s="13" t="n">
         <v>8000</v>
@@ -15266,10 +15236,10 @@
         </is>
       </c>
       <c r="G312" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H312" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I312" s="17" t="n">
         <v>8000</v>
@@ -15311,10 +15281,10 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H313" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I313" s="13" t="n">
         <v>8000</v>
@@ -15356,10 +15326,10 @@
         </is>
       </c>
       <c r="G314" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H314" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I314" s="17" t="n">
         <v>8000</v>
@@ -15401,10 +15371,10 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H315" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I315" s="13" t="n">
         <v>8000</v>
@@ -15446,10 +15416,10 @@
         </is>
       </c>
       <c r="G316" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H316" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I316" s="17" t="n">
         <v>8000</v>
@@ -15536,10 +15506,10 @@
         </is>
       </c>
       <c r="G318" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H318" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I318" s="17" t="n">
         <v>8000</v>
@@ -15581,10 +15551,10 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H319" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I319" s="13" t="n">
         <v>8000</v>
@@ -15626,10 +15596,10 @@
         </is>
       </c>
       <c r="G320" s="14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H320" s="16" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I320" s="17" t="n">
         <v>8000</v>
@@ -15671,10 +15641,10 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H321" s="6" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I321" s="13" t="n">
         <v>8000</v>
@@ -15758,13 +15728,13 @@
         <v>105</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>13911000</v>
+        <v>11979000</v>
       </c>
       <c r="D3" t="n">
         <v>32.9</v>
       </c>
       <c r="E3" t="n">
-        <v>30.8</v>
+        <v>33.5</v>
       </c>
     </row>
     <row r="4">
@@ -15777,13 +15747,13 @@
         <v>47</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>8573000</v>
+        <v>5445000</v>
       </c>
       <c r="D4" t="n">
         <v>14.7</v>
       </c>
       <c r="E4" t="n">
-        <v>19</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="5">
@@ -15796,13 +15766,13 @@
         <v>35</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>5573000</v>
+        <v>3445000</v>
       </c>
       <c r="D5" t="n">
         <v>11</v>
       </c>
       <c r="E5" t="n">
-        <v>12.3</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="6">
@@ -15815,13 +15785,13 @@
         <v>59</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>7219000</v>
+        <v>7176000</v>
       </c>
       <c r="D6" t="n">
         <v>18.5</v>
       </c>
       <c r="E6" t="n">
-        <v>16</v>
+        <v>20.1</v>
       </c>
     </row>
     <row r="7">
@@ -15834,13 +15804,13 @@
         <v>61</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>8600000</v>
+        <v>6633000</v>
       </c>
       <c r="D7" t="n">
         <v>19.1</v>
       </c>
       <c r="E7" t="n">
-        <v>19</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="8">
@@ -15853,13 +15823,13 @@
         <v>12</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1273000</v>
+        <v>1030000</v>
       </c>
       <c r="D8" t="n">
         <v>3.8</v>
       </c>
       <c r="E8" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="9">
@@ -15872,7 +15842,7 @@
         <v>319</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>45149000</v>
+        <v>35708000</v>
       </c>
     </row>
   </sheetData>
@@ -15886,7 +15856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -15935,16 +15905,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>96</v>
       </c>
       <c r="C3" s="6" t="n">
         <v>73000</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>949000</v>
+        <v>7008000</v>
       </c>
       <c r="E3" t="n">
-        <v>4.1</v>
+        <v>30.1</v>
       </c>
     </row>
     <row r="4">
@@ -15952,16 +15922,16 @@
         <v>12</v>
       </c>
       <c r="B4" t="n">
-        <v>182</v>
+        <v>95</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>100000</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>18200000</v>
+        <v>9500000</v>
       </c>
       <c r="E4" t="n">
-        <v>57.1</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="5">
@@ -15969,63 +15939,29 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>31</v>
+        <v>128</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>150000</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>4650000</v>
+        <v>19200000</v>
       </c>
       <c r="E5" t="n">
-        <v>9.699999999999999</v>
+        <v>40.1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>30</v>
-      </c>
-      <c r="B6" t="n">
-        <v>38</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>7600000</v>
-      </c>
-      <c r="E6" t="n">
-        <v>11.9</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>50</v>
-      </c>
-      <c r="B7" t="n">
-        <v>55</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>250000</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>13750000</v>
-      </c>
-      <c r="E7" t="n">
-        <v>17.2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B6" s="4" t="n">
         <v>319</v>
       </c>
-      <c r="D8" s="7" t="n">
-        <v>45149000</v>
+      <c r="D6" s="7" t="n">
+        <v>35708000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>